<commit_message>
Add Full address with Unit
</commit_message>
<xml_diff>
--- a/LW_Web/_Templates/_Template - Tenant_Arrears.xlsx
+++ b/LW_Web/_Templates/_Template - Tenant_Arrears.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vincent\Source\Repos\lemlewolff\LW_Web\_Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E677545-1994-4F5A-827A-83CECC2D4998}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9A7B974-082B-4CDB-BB32-E9453807A74A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="212" xr2:uid="{6455282C-9733-4B18-88B6-55E0A49963C2}"/>
+    <workbookView xWindow="2070" yWindow="780" windowWidth="24060" windowHeight="13485" tabRatio="212" xr2:uid="{6455282C-9733-4B18-88B6-55E0A49963C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$12:$W$12</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="64">
   <si>
     <t>Legend</t>
   </si>
@@ -47,9 +50,6 @@
     <t>Current Progress</t>
   </si>
   <si>
-    <t>Category</t>
-  </si>
-  <si>
     <t>Description</t>
   </si>
   <si>
@@ -200,15 +200,9 @@
     <t>Expired Lease</t>
   </si>
   <si>
-    <t>ABC</t>
-  </si>
-  <si>
     <t>Last Note &gt; 45 Days</t>
   </si>
   <si>
-    <t>KEY</t>
-  </si>
-  <si>
     <t>Tenant Yardi ID</t>
   </si>
   <si>
@@ -225,13 +219,25 @@
   </si>
   <si>
     <t>Is Resolved From Prior Snapshot</t>
+  </si>
+  <si>
+    <t>Full Address</t>
+  </si>
+  <si>
+    <t>Indicator</t>
+  </si>
+  <si>
+    <t>red fill</t>
+  </si>
+  <si>
+    <t>Bold Red</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -271,9 +277,14 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color theme="0"/>
+      <color rgb="FF69472D"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -281,20 +292,21 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFA80000"/>
+      <color rgb="FFC00000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF69472D"/>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FFC00000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -333,12 +345,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF006080"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -350,7 +356,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -480,17 +486,6 @@
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
@@ -570,11 +565,73 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="2" tint="-0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="2" tint="-0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="2" tint="-0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -597,9 +654,6 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="3" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -617,9 +671,6 @@
     </xf>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -646,9 +697,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -670,21 +718,39 @@
     <xf numFmtId="14" fontId="1" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -694,62 +760,113 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1113,441 +1230,454 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D3D621A-9594-4DC5-BEAB-55FA428C4FC8}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:V13"/>
+  <dimension ref="A1:W13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.85546875" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" customWidth="1"/>
-    <col min="5" max="5" width="37.140625" customWidth="1"/>
-    <col min="6" max="6" width="10.7109375" customWidth="1"/>
-    <col min="7" max="7" width="22.28515625" style="21" customWidth="1"/>
-    <col min="8" max="8" width="19.5703125" style="26" customWidth="1"/>
-    <col min="9" max="9" width="9.85546875" style="21" customWidth="1"/>
-    <col min="10" max="10" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.140625" style="21"/>
-    <col min="12" max="12" width="8.140625" style="21" customWidth="1"/>
-    <col min="13" max="13" width="9.85546875" style="21" customWidth="1"/>
-    <col min="14" max="14" width="22.85546875" customWidth="1"/>
-    <col min="15" max="15" width="12.42578125" customWidth="1"/>
-    <col min="16" max="17" width="13" customWidth="1"/>
-    <col min="18" max="18" width="10.7109375" style="36" customWidth="1"/>
-    <col min="19" max="20" width="14.5703125" customWidth="1"/>
-    <col min="21" max="21" width="17.85546875" customWidth="1"/>
-    <col min="22" max="22" width="12.7109375" customWidth="1"/>
+    <col min="1" max="1" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.28515625" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" customWidth="1"/>
+    <col min="4" max="4" width="12.85546875" customWidth="1"/>
+    <col min="5" max="5" width="51.7109375" customWidth="1"/>
+    <col min="6" max="6" width="33" customWidth="1"/>
+    <col min="7" max="7" width="14.140625" customWidth="1"/>
+    <col min="8" max="8" width="22.28515625" style="19" customWidth="1"/>
+    <col min="9" max="9" width="19.5703125" style="23" customWidth="1"/>
+    <col min="10" max="10" width="9.85546875" style="19" customWidth="1"/>
+    <col min="11" max="11" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.42578125" style="19" customWidth="1"/>
+    <col min="13" max="13" width="12.7109375" style="19" customWidth="1"/>
+    <col min="14" max="14" width="11.42578125" style="19" customWidth="1"/>
+    <col min="15" max="15" width="22.85546875" customWidth="1"/>
+    <col min="16" max="16" width="12.42578125" customWidth="1"/>
+    <col min="17" max="18" width="13" customWidth="1"/>
+    <col min="19" max="19" width="10.7109375" style="30" customWidth="1"/>
+    <col min="20" max="21" width="14.5703125" customWidth="1"/>
+    <col min="22" max="22" width="17.85546875" customWidth="1"/>
+    <col min="23" max="23" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22">
-      <c r="A1" s="47" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48" t="s">
+    <row r="1" spans="1:23">
+      <c r="A1" s="44" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48" t="s">
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
+      <c r="H1" s="69" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="48"/>
-      <c r="J1" s="48"/>
+      <c r="I1" s="37"/>
+      <c r="J1" s="37"/>
       <c r="K1" s="1"/>
-      <c r="L1" s="5"/>
+      <c r="M1" s="5"/>
     </row>
-    <row r="2" spans="1:22">
-      <c r="A2" s="49" t="s">
+    <row r="2" spans="1:23">
+      <c r="A2" s="45" t="s">
+        <v>61</v>
+      </c>
+      <c r="B2" s="46"/>
+      <c r="C2" s="67" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="50" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="51"/>
+      <c r="D2" s="68"/>
       <c r="E2" s="3" t="s">
         <v>1</v>
       </c>
       <c r="F2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="27" t="s">
+      <c r="I2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="K2" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="42" t="s">
+      <c r="M2" s="5"/>
+    </row>
+    <row r="3" spans="1:23">
+      <c r="A3" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="5"/>
-      <c r="M2" s="52" t="s">
-        <v>56</v>
-      </c>
-      <c r="N2" s="52"/>
+      <c r="B3" s="40"/>
+      <c r="C3" s="56" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="57"/>
+      <c r="E3" s="33" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="4">
+        <f>COUNTIFS(G13:G999227, "&lt;=5000")</f>
+        <v>0</v>
+      </c>
+      <c r="G3" s="8">
+        <f>SUMIFS(G13:G999227, G13:G999227, "&lt;=5000")</f>
+        <v>0</v>
+      </c>
+      <c r="H3" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="I3" s="4">
+        <f>COUNTIFS(L13:L999227, "LKEM", H13:H999227, "&lt;&gt;")</f>
+        <v>0</v>
+      </c>
+      <c r="J3" s="4">
+        <f>COUNTIFS(L13:L999227, "Horing", H13:H999227, "&lt;&gt;")</f>
+        <v>0</v>
+      </c>
+      <c r="K3" s="38"/>
+      <c r="M3" s="20"/>
     </row>
-    <row r="3" spans="1:22">
-      <c r="A3" s="53" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" s="54"/>
-      <c r="C3" s="54" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="55"/>
-      <c r="E3" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="4">
-        <f>COUNTIFS(F13:F999227, "&lt;=5000")</f>
-        <v>0</v>
-      </c>
-      <c r="G3" s="9">
-        <f>SUMIFS(F13:F999227, F13:F999227, "&lt;=5000")</f>
-        <v>0</v>
-      </c>
-      <c r="H3" s="28" t="s">
+    <row r="4" spans="1:23">
+      <c r="A4" s="74" t="s">
         <v>14</v>
       </c>
-      <c r="I3" s="4">
-        <f>COUNTIFS(K13:K999227, "LKEM", G13:G999227, "&lt;&gt;")</f>
-        <v>0</v>
-      </c>
-      <c r="J3" s="4">
-        <f>COUNTIFS(K13:K999227, "Horing", G13:G999227, "&lt;&gt;")</f>
-        <v>0</v>
-      </c>
-      <c r="K3" s="42"/>
-      <c r="L3" s="22"/>
-      <c r="M3" s="33"/>
-      <c r="N3" s="34" t="s">
-        <v>53</v>
-      </c>
+      <c r="B4" s="75"/>
+      <c r="C4" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="73"/>
+      <c r="E4" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" s="5">
+        <f>COUNTIFS(G13:G999227, "&gt;5000", G13:G999227, "&lt;=10000")</f>
+        <v>0</v>
+      </c>
+      <c r="G4" s="6">
+        <f>SUMIFS(G13:G999227, G13:G999227, "&gt;5000", G13:G999227, "&lt;=10000")</f>
+        <v>0</v>
+      </c>
+      <c r="H4" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="I4" s="5">
+        <f>COUNTIFS(L13:L999227, "LKEM", J13:J999227, "&gt;30")</f>
+        <v>0</v>
+      </c>
+      <c r="J4" s="5">
+        <f>COUNTIFS(L13:L999227, "horing", J13:J999227, "&gt;30")</f>
+        <v>0</v>
+      </c>
+      <c r="K4" s="38"/>
+      <c r="M4" s="21"/>
     </row>
-    <row r="4" spans="1:22">
-      <c r="A4" s="44" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" s="45"/>
-      <c r="C4" s="45" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="46"/>
-      <c r="E4" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="F4" s="5">
-        <f>COUNTIFS(F13:F999227, "&gt;5000", F13:F999227, "&lt;=10000")</f>
-        <v>0</v>
-      </c>
-      <c r="G4" s="6">
-        <f>SUMIFS(F13:F999227, F13:F999227, "&gt;5000", F13:F999227, "&lt;=10000")</f>
-        <v>0</v>
-      </c>
-      <c r="H4" s="29" t="s">
+    <row r="5" spans="1:23">
+      <c r="A5" s="60" t="s">
         <v>18</v>
       </c>
-      <c r="I4" s="5">
-        <f>COUNTIFS(K13:K999227, "LKEM", I13:I999227, "&gt;30")</f>
-        <v>0</v>
-      </c>
-      <c r="J4" s="5">
-        <f>COUNTIFS(K13:K999227, "horing", I13:I999227, "&gt;30")</f>
-        <v>0</v>
-      </c>
-      <c r="K4" s="42"/>
-      <c r="L4" s="23"/>
-      <c r="M4" s="35" t="s">
-        <v>54</v>
-      </c>
-      <c r="N4" s="34" t="s">
-        <v>55</v>
-      </c>
+      <c r="B5" s="71"/>
+      <c r="C5" s="70" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="53"/>
+      <c r="E5" s="35" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" s="7">
+        <f>COUNTIFS(G13:G999227, "&gt;10000", G13:G999227, "&lt;=20000")</f>
+        <v>0</v>
+      </c>
+      <c r="G5" s="8">
+        <f>SUMIFS(G13:G999227, G13:G999227, "&gt;10000", G13:G999227, "&lt;=20000")</f>
+        <v>0</v>
+      </c>
+      <c r="H5" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="I5" s="4">
+        <f>COUNTIFS(L13:L999227, "LKEM", H13:H999227, "Closed")</f>
+        <v>0</v>
+      </c>
+      <c r="J5" s="4">
+        <f>COUNTIFS(L13:L999227, "Horing", H13:H999227, "closed")</f>
+        <v>0</v>
+      </c>
+      <c r="K5" s="38"/>
+      <c r="M5" s="21"/>
     </row>
-    <row r="5" spans="1:22">
-      <c r="A5" s="38" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" s="39"/>
-      <c r="C5" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" s="40"/>
-      <c r="E5" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="F5" s="7">
-        <f>COUNTIFS(F13:F999227, "&gt;10000", F13:F999227, "&lt;=20000")</f>
-        <v>0</v>
-      </c>
-      <c r="G5" s="9">
-        <f>SUMIFS(F13:F999227, F13:F999227, "&gt;10000", F13:F999227, "&lt;=20000")</f>
-        <v>0</v>
-      </c>
-      <c r="H5" s="30" t="s">
+    <row r="6" spans="1:23">
+      <c r="A6" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="I5" s="4">
-        <f>COUNTIFS(K13:K999227, "LKEM", G13:G999227, "Closed")</f>
-        <v>0</v>
-      </c>
-      <c r="J5" s="4">
-        <f>COUNTIFS(K13:K999227, "Horing", G13:G999227, "closed")</f>
-        <v>0</v>
-      </c>
-      <c r="K5" s="42"/>
-      <c r="L5" s="23"/>
-    </row>
-    <row r="6" spans="1:22">
-      <c r="A6" s="44" t="s">
+      <c r="B6" s="59"/>
+      <c r="C6" s="54" t="s">
         <v>23</v>
       </c>
-      <c r="B6" s="45"/>
-      <c r="C6" s="45" t="s">
+      <c r="D6" s="55"/>
+      <c r="E6" s="34" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="46"/>
-      <c r="E6" s="5" t="s">
-        <v>25</v>
-      </c>
       <c r="F6" s="5">
-        <f>COUNTIFS(F13:F999227, "&gt;20000", F13:F999227, "&lt;=30000")</f>
+        <f>COUNTIFS(G13:G999227, "&gt;20000", G13:G999227, "&lt;=30000")</f>
         <v>0</v>
       </c>
       <c r="G6" s="6">
-        <f>SUMIFS(F13:F999227, F13:F999227, "&gt;20000", F13:F999227, "&lt;=30000")</f>
-        <v>0</v>
-      </c>
-      <c r="H6" s="29"/>
+        <f>SUMIFS(G13:G999227, G13:G999227, "&gt;20000", G13:G999227, "&lt;=30000")</f>
+        <v>0</v>
+      </c>
+      <c r="H6" s="26"/>
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
-      <c r="K6" s="42"/>
-      <c r="L6" s="23"/>
+      <c r="K6" s="38"/>
+      <c r="M6" s="21"/>
     </row>
-    <row r="7" spans="1:22">
-      <c r="A7" s="38" t="s">
+    <row r="7" spans="1:23">
+      <c r="A7" s="60" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="61"/>
+      <c r="C7" s="52" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="53"/>
+      <c r="E7" s="35" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" s="9">
+        <f>COUNTIFS(G13:G999227, "&gt;30000", G13:G999227, "&lt;=40000")</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="10">
+        <f>SUMIFS(G13:G999227, G13:G999227, "&gt;30000", G13:G999227, "&lt;=40000")</f>
+        <v>0</v>
+      </c>
+      <c r="H7" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="I7" s="11">
+        <f>I3-I4</f>
+        <v>0</v>
+      </c>
+      <c r="J7" s="11">
+        <f>J3-J4</f>
+        <v>0</v>
+      </c>
+      <c r="K7" s="50" t="s">
+        <v>28</v>
+      </c>
+      <c r="M7" s="21"/>
+    </row>
+    <row r="8" spans="1:23">
+      <c r="A8" s="78" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="39"/>
-      <c r="C7" s="39" t="s">
-        <v>26</v>
-      </c>
-      <c r="D7" s="40"/>
-      <c r="E7" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="10">
-        <f>COUNTIFS(F13:F999227, "&gt;30000", F13:F999227, "&lt;=40000")</f>
-        <v>0</v>
-      </c>
-      <c r="G7" s="11">
-        <f>SUMIFS(F13:F999227, F13:F999227, "&gt;30000", F13:F999227, "&lt;=40000")</f>
-        <v>0</v>
-      </c>
-      <c r="H7" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="I7" s="12">
-        <f>I3-I4</f>
-        <v>0</v>
-      </c>
-      <c r="J7" s="12">
-        <f>J3-J4</f>
-        <v>0</v>
-      </c>
-      <c r="K7" s="41" t="s">
+      <c r="B8" s="79"/>
+      <c r="C8" s="72" t="s">
         <v>29</v>
       </c>
-      <c r="L7" s="23"/>
-    </row>
-    <row r="8" spans="1:22">
-      <c r="A8" s="44" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="45"/>
-      <c r="C8" s="45" t="s">
+      <c r="D8" s="73"/>
+      <c r="E8" s="34" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="46"/>
-      <c r="E8" s="5" t="s">
+      <c r="F8" s="5">
+        <f>COUNTIFS(G13:G999227, "&gt;40000", G13:G999227, "&lt;=50000")</f>
+        <v>0</v>
+      </c>
+      <c r="G8" s="12">
+        <f>SUMIFS(G13:G999227, G13:G999227, "&gt;40000", G13:G999227, "&lt;=50000")</f>
+        <v>0</v>
+      </c>
+      <c r="H8" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="F8" s="5">
-        <f>COUNTIFS(F13:F999227, "&gt;40000", F13:F999227, "&lt;=50000")</f>
-        <v>0</v>
-      </c>
-      <c r="G8" s="13">
-        <f>SUMIFS(F13:F999227, F13:F999227, "&gt;40000", F13:F999227, "&lt;=50000")</f>
-        <v>0</v>
-      </c>
-      <c r="H8" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="I8" s="14" t="e">
+      <c r="I8" s="13" t="e">
         <f>ROUND(I7/I3, 2)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="J8" s="14" t="e">
+      <c r="J8" s="13" t="e">
         <f>ROUND(J7/J3, 2)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="K8" s="42"/>
-      <c r="L8" s="5"/>
+      <c r="K8" s="38"/>
+      <c r="M8" s="5"/>
     </row>
-    <row r="9" spans="1:22">
-      <c r="A9" s="38"/>
-      <c r="B9" s="39"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="7" t="s">
-        <v>33</v>
+    <row r="9" spans="1:23">
+      <c r="A9" s="77" t="s">
+        <v>62</v>
+      </c>
+      <c r="B9" s="77"/>
+      <c r="C9" s="62" t="s">
+        <v>52</v>
+      </c>
+      <c r="D9" s="76"/>
+      <c r="E9" s="66" t="s">
+        <v>32</v>
       </c>
       <c r="F9" s="7">
-        <f>COUNTIFS(F13:F999227, "&gt;50000", F13:F999227, "&lt;100000")</f>
-        <v>0</v>
-      </c>
-      <c r="G9" s="9">
-        <f>SUMIFS(F13:F999227, F13:F999227, "&gt;50000", F13:F999227, "&lt;100000")</f>
-        <v>0</v>
-      </c>
-      <c r="H9" s="30"/>
+        <f>COUNTIFS(G13:G999227, "&gt;50000", G13:G999227, "&lt;100000")</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="8">
+        <f>SUMIFS(G13:G999227, G13:G999227, "&gt;50000", G13:G999227, "&lt;100000")</f>
+        <v>0</v>
+      </c>
+      <c r="H9" s="27"/>
       <c r="I9" s="7"/>
       <c r="J9" s="7"/>
-      <c r="K9" s="42"/>
-      <c r="L9" s="5"/>
+      <c r="K9" s="38"/>
+      <c r="M9" s="5"/>
     </row>
-    <row r="10" spans="1:22">
-      <c r="A10" s="44"/>
-      <c r="B10" s="45"/>
-      <c r="C10" s="45"/>
-      <c r="D10" s="46"/>
-      <c r="E10" s="5" t="s">
-        <v>34</v>
+    <row r="10" spans="1:23">
+      <c r="A10" s="63" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" s="63"/>
+      <c r="C10" s="64" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10" s="65"/>
+      <c r="E10" s="34" t="s">
+        <v>33</v>
       </c>
       <c r="F10" s="5">
-        <f>COUNTIFS(F13:F999227, "&gt;=100000")</f>
+        <f>COUNTIFS(G13:G999227, "&gt;=100000")</f>
         <v>0</v>
       </c>
       <c r="G10" s="6">
-        <f>SUMIFS(F13:F999227, F13:F999227, "&gt;=100000")</f>
-        <v>0</v>
-      </c>
-      <c r="H10" s="29"/>
+        <f>SUMIFS(G13:G999227, G13:G999227, "&gt;=100000")</f>
+        <v>0</v>
+      </c>
+      <c r="H10" s="26"/>
       <c r="I10" s="5"/>
       <c r="J10" s="5"/>
-      <c r="K10" s="42"/>
-      <c r="L10" s="5"/>
+      <c r="K10" s="38"/>
+      <c r="M10" s="5"/>
     </row>
-    <row r="11" spans="1:22">
-      <c r="A11" s="38"/>
-      <c r="B11" s="39"/>
-      <c r="C11" s="39"/>
-      <c r="D11" s="40"/>
-      <c r="E11" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="F11" s="16">
+    <row r="11" spans="1:23">
+      <c r="A11" s="41"/>
+      <c r="B11" s="42"/>
+      <c r="C11" s="42"/>
+      <c r="D11" s="43"/>
+      <c r="E11" s="36" t="s">
+        <v>34</v>
+      </c>
+      <c r="F11" s="14">
         <f>SUM(F3:F10)</f>
         <v>0</v>
       </c>
-      <c r="G11" s="17">
+      <c r="G11" s="15">
         <f>SUM(G3:G10)</f>
         <v>0</v>
       </c>
-      <c r="H11" s="30"/>
+      <c r="H11" s="27"/>
       <c r="I11" s="7"/>
       <c r="J11" s="7"/>
-      <c r="K11" s="43"/>
-      <c r="L11" s="5"/>
-      <c r="R11" s="56" t="s">
-        <v>61</v>
-      </c>
-      <c r="S11" s="57"/>
-      <c r="T11" s="57"/>
-      <c r="U11" s="57"/>
-      <c r="V11" s="58"/>
+      <c r="K11" s="51"/>
+      <c r="M11" s="5"/>
+      <c r="S11" s="47" t="s">
+        <v>58</v>
+      </c>
+      <c r="T11" s="48"/>
+      <c r="U11" s="48"/>
+      <c r="V11" s="48"/>
+      <c r="W11" s="49"/>
     </row>
-    <row r="12" spans="1:22" ht="30" customHeight="1">
-      <c r="A12" s="18" t="s">
+    <row r="12" spans="1:23" ht="30" customHeight="1">
+      <c r="A12" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="C12" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="D12" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="D12" s="19" t="s">
+      <c r="E12" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="F12" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="E12" s="18" t="s">
+      <c r="G12" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="F12" s="19" t="s">
+      <c r="H12" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="G12" s="19" t="s">
+      <c r="I12" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="H12" s="32" t="s">
+      <c r="J12" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="I12" s="19" t="s">
+      <c r="K12" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="J12" s="20" t="s">
+      <c r="L12" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="M12" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="K12" s="24" t="s">
+      <c r="N12" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="O12" s="22" t="s">
+        <v>47</v>
+      </c>
+      <c r="P12" s="22" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q12" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="L12" s="25" t="s">
-        <v>46</v>
-      </c>
-      <c r="M12" s="25" t="s">
-        <v>47</v>
-      </c>
-      <c r="N12" s="25" t="s">
-        <v>48</v>
-      </c>
-      <c r="O12" s="25" t="s">
-        <v>49</v>
-      </c>
-      <c r="P12" s="25" t="s">
+      <c r="R12" s="31" t="s">
         <v>51</v>
       </c>
-      <c r="Q12" s="37" t="s">
-        <v>52</v>
-      </c>
-      <c r="R12" s="59" t="s">
+      <c r="S12" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="T12" s="32" t="s">
+        <v>55</v>
+      </c>
+      <c r="U12" s="32" t="s">
+        <v>56</v>
+      </c>
+      <c r="V12" s="32" t="s">
+        <v>59</v>
+      </c>
+      <c r="W12" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="S12" s="59" t="s">
-        <v>58</v>
-      </c>
-      <c r="T12" s="59" t="s">
-        <v>59</v>
-      </c>
-      <c r="U12" s="59" t="s">
-        <v>62</v>
-      </c>
-      <c r="V12" s="59" t="s">
-        <v>60</v>
-      </c>
     </row>
-    <row r="13" spans="1:22">
-      <c r="Q13" s="26"/>
+    <row r="13" spans="1:23">
+      <c r="R13" s="23"/>
     </row>
   </sheetData>
+  <autoFilter ref="A12:W12" xr:uid="{2D3D621A-9594-4DC5-BEAB-55FA428C4FC8}"/>
   <mergeCells count="26">
-    <mergeCell ref="M2:N2"/>
+    <mergeCell ref="S11:W11"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="K7:K11"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="E1:G1"/>
+    <mergeCell ref="H1:J1"/>
     <mergeCell ref="K2:K6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:D3"/>
@@ -1558,28 +1688,15 @@
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="E1:G1"/>
-    <mergeCell ref="H1:J1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
-    <mergeCell ref="R11:V11"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="K7:K11"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="C11:D11"/>
   </mergeCells>
-  <conditionalFormatting sqref="A13:Q9227">
+  <conditionalFormatting sqref="A13:R9227">
     <cfRule type="expression" dxfId="1" priority="1">
-      <formula>AND($I13&lt;&gt;"",$I13&gt;45)</formula>
+      <formula>AND($J13&lt;&gt;"",$J13&gt;45)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="0" priority="2">
-      <formula>AND($Q13&lt;TODAY(),$B13&lt;&gt;"")</formula>
+      <formula>AND($R13&lt;TODAY(),$B13&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>